<commit_message>
feat(F-NAR-016): TREE-DIF-071 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-071.xlsx
+++ b/stories/arbres/TREE-DIF-071.xlsx
@@ -16467,7 +16467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -16510,6 +16510,20 @@
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>

<commit_message>
feat(F-NAR-019): TREE-DIF-071 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-071.xlsx
+++ b/stories/arbres/TREE-DIF-071.xlsx
@@ -5329,17 +5329,17 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Le pli blanc tremble vers la porte. Près du battant, le vent pousse, fort. Mila lève le papier, trop tôt. J'ouvre, trop vite ! Le papier part de travers, pris. Le vent l'a pris ! Le battant claque, trop large. Ici, ça souffle trop. Il lui faut un air plus calme. Alors on fait comment ? Tu vois comment, avec lui ?</t>
+          <t>Le pli blanc tremble vers la porte. Près du battant, le vent pousse, fort. Mila lève le papier, trop tôt. J'ouvre, trop vite ! Le papier part de travers, pris. Le vent l'a pris ! Le battant claque, trop large. Ici, ça souffle trop. Sans le vent, le papier irait droit. Alors on fait comment ? Tu vois comment, avec lui ?</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Le pli blanc tremble vers la porte. Près du battant, le &lt;emphasis level="moderate"&gt;vent&lt;/emphasis&gt; pousse, fort. Mila lève le papier, trop tôt. J'ouvre, trop vite ! Le papier part de travers, pris. Le vent l'a pris ! Le battant claque, trop large. Ici, ça souffle trop. Il lui faut un air plus calme. Alors on fait comment ? Tu vois comment, avec lui ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Le pli blanc tremble vers la porte. Près du battant, le &lt;emphasis level="moderate"&gt;vent&lt;/emphasis&gt; pousse, fort. Mila lève le papier, trop tôt. J'ouvre, trop vite ! Le papier part de travers, pris. Le vent l'a pris ! Le battant claque, trop large. Ici, ça souffle trop. Sans le vent, le papier irait droit. Alors on fait comment ? Tu vois comment, avec lui ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Le pli blanc tremble vers la porte. Près du battant, le &lt;emphasis&gt;vent&lt;/emphasis&gt; pousse, fort. Mila lève le papier, trop tôt. J'ouvre, trop vite ! Le papier part de travers, pris. Le vent l'a pris ! Le battant claque, trop large. Ici, ça souffle trop. Il lui faut un air plus calme. Alors on fait comment ? Tu vois comment, avec lui ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Le pli blanc tremble vers la porte. Près du battant, le &lt;emphasis&gt;vent&lt;/emphasis&gt; pousse, fort. Mila lève le papier, trop tôt. J'ouvre, trop vite ! Le papier part de travers, pris. Le vent l'a pris ! Le battant claque, trop large. Ici, ça souffle trop. Sans le vent, le papier irait droit. Alors on fait comment ? Tu vois comment, avec lui ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr"/>
@@ -5485,7 +5485,7 @@
 enfant-f|Le vent l'a pris !
 narrateur|Le battant claque, trop large.
 papa|Ici, ça souffle trop.
-maman|Il lui faut un air plus calme.
+maman|Sans le vent, le papier irait droit.
 enfant-f|Alors on fait comment ?
 papa|Tu vois comment, avec lui ?</t>
         </is>
@@ -8149,17 +8149,17 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Le nez lourd glisse entre les rayons, libre. Tu as tenu le guidon, loin du métal. La roue n'a plus attrapé le nez. Tes mains ont laissé le nez passer. On rentre, essuie le trombone. Le trombone reste froid, contre le nez. Le trombone reste froid, contre le nez plié.</t>
+          <t>Le nez lourd glisse entre les rayons, libre. Tu as tenu le guidon, loin du métal. La roue n'a plus attrapé le nez. Tes mains ont laissé le nez passer. On rentre, essuie le trombone. Le trombone brille un peu, contre le papier. Le trombone reste froid, contre le nez plié.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le nez lourd glisse entre les rayons, libre. Tu as tenu le &lt;emphasis level="moderate"&gt;guidon&lt;/emphasis&gt;, loin du métal. La roue n'a plus attrapé le nez. Tes mains ont laissé le nez passer. On rentre, essuie le trombone. Le trombone reste froid, contre le nez. Le trombone reste froid, contre le nez plié.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le nez lourd glisse entre les rayons, libre. Tu as tenu le &lt;emphasis level="moderate"&gt;guidon&lt;/emphasis&gt;, loin du métal. La roue n'a plus attrapé le nez. Tes mains ont laissé le nez passer. On rentre, essuie le trombone. Le trombone brille un peu, contre le papier. Le trombone reste froid, contre le nez plié.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le nez lourd glisse entre les rayons, libre. Tu as tenu le &lt;emphasis&gt;guidon&lt;/emphasis&gt;, loin du métal. La roue n'a plus attrapé le nez. Tes mains ont laissé le nez passer. On rentre, essuie le trombone. Le trombone reste froid, contre le nez. Le trombone reste froid, contre le nez plié.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le nez lourd glisse entre les rayons, libre. Tu as tenu le &lt;emphasis&gt;guidon&lt;/emphasis&gt;, loin du métal. La roue n'a plus attrapé le nez. Tes mains ont laissé le nez passer. On rentre, essuie le trombone. Le trombone brille un peu, contre le papier. Le trombone reste froid, contre le nez plié.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr"/>
@@ -8302,7 +8302,7 @@
 enfant-m|La roue n'a plus attrapé le nez.
 papa|Tes mains ont laissé le nez passer.
 maman|On rentre, essuie le trombone.
-narrateur|Le trombone reste froid, contre le nez.
+narrateur|Le trombone brille un peu, contre le papier.
 narrateur|Le trombone reste froid, contre le nez plié.</t>
         </is>
       </c>
@@ -10566,17 +10566,17 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Le nez trop lourd penche vers le seuil. Près de la porte, le vent pousse, large. Mila lève le trombone, trop tôt. Je tiens le battant, ouvert ! Le nez trop lourd plonge, trop vite. Il est tombé près du seuil ! Le papier file de côté, trop loin. Ici, le vent plus le poids, ça plonge. Il lui faut un air plus calme. Alors on fait comment ? Tu vois comment, avec lui ?</t>
+          <t>Le nez trop lourd penche vers le seuil. Près de la porte, le vent pousse, large. Mila lève le trombone, trop tôt. Je tiens le battant, ouvert ! Le nez trop lourd plonge, trop vite. Il est tombé près du seuil ! Le papier file de côté, trop loin. Ici, le vent fait plonger le nez. Le nez a besoin d'un battant fermé. Alors on fait comment ? Tu vois comment, avec lui ?</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Le nez trop lourd penche vers le seuil. Près de la porte, le &lt;emphasis level="moderate"&gt;vent&lt;/emphasis&gt; pousse, large. Mila lève le trombone, trop tôt. Je tiens le battant, ouvert ! Le nez trop lourd plonge, trop vite. Il est tombé près du seuil ! Le papier file de côté, trop loin. Ici, le vent plus le poids, ça plonge. Il lui faut un air plus calme. Alors on fait comment ? Tu vois comment, avec lui ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Le nez trop lourd penche vers le seuil. Près de la porte, le &lt;emphasis level="moderate"&gt;vent&lt;/emphasis&gt; pousse, large. Mila lève le trombone, trop tôt. Je tiens le battant, ouvert ! Le nez trop lourd plonge, trop vite. Il est tombé près du seuil ! Le papier file de côté, trop loin. Ici, le vent fait plonger le nez. Le nez a besoin d'un battant fermé. Alors on fait comment ? Tu vois comment, avec lui ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Le nez trop lourd penche vers le seuil. Près de la porte, le &lt;emphasis&gt;vent&lt;/emphasis&gt; pousse, large. Mila lève le trombone, trop tôt. Je tiens le battant, ouvert ! Le nez trop lourd plonge, trop vite. Il est tombé près du seuil ! Le papier file de côté, trop loin. Ici, le vent plus le poids, ça plonge. Il lui faut un air plus calme. Alors on fait comment ? Tu vois comment, avec lui ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Le nez trop lourd penche vers le seuil. Près de la porte, le &lt;emphasis&gt;vent&lt;/emphasis&gt; pousse, large. Mila lève le trombone, trop tôt. Je tiens le battant, ouvert ! Le nez trop lourd plonge, trop vite. Il est tombé près du seuil ! Le papier file de côté, trop loin. Ici, le vent fait plonger le nez. Le nez a besoin d'un battant fermé. Alors on fait comment ? Tu vois comment, avec lui ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr"/>
@@ -10721,8 +10721,8 @@
 narrateur|Le nez trop lourd plonge, trop vite.
 enfant-f|Il est tombé près du seuil !
 narrateur|Le papier file de côté, trop loin.
-papa|Ici, le vent plus le poids, ça plonge.
-maman|Il lui faut un air plus calme.
+papa|Ici, le vent fait plonger le nez.
+maman|Le nez a besoin d'un battant fermé.
 enfant-f|Alors on fait comment ?
 papa|Tu vois comment, avec lui ?</t>
         </is>
@@ -13386,17 +13386,17 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Le long du blanc, l'avion glisse jusqu'à la porte. Tu as tenu, j'ai tracé. Le pneu n'a plus mangé la piste. Tes mains ont laissé la piste. On rentre, essuie tes doigts blancs. Un trait de craie sèche sur le ciment. Un trait de craie sèche sur le ciment, net.</t>
+          <t>Le long du blanc, l'avion glisse jusqu'à la porte. Tu as tenu, j'ai tracé. Le pneu n'a plus mangé la piste. Tes mains ont laissé la piste. On rentre, essuie tes doigts blancs. Un trait de craie sèche sous les guidons. Un trait de craie sèche sur le ciment, net.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le long du blanc, l'avion glisse jusqu'à la porte. Tu as tenu, j'ai tracé. Le pneu n'a plus mangé la piste. Tes mains ont laissé la piste. On rentre, essuie tes doigts blancs. Un trait de craie sèche sur le ciment. Un trait de craie sèche sur le ciment, net.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le long du blanc, l'avion glisse jusqu'à la porte. Tu as tenu, j'ai tracé. Le pneu n'a plus mangé la piste. Tes mains ont laissé la piste. On rentre, essuie tes doigts blancs. Un trait de craie sèche sous les &lt;emphasis level="moderate"&gt;guidon&lt;/emphasis&gt;s. Un trait de craie sèche sur le ciment, net.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le long du blanc, l'avion glisse jusqu'à la porte. Tu as tenu, j'ai tracé. Le pneu n'a plus mangé la piste. Tes mains ont laissé la piste. On rentre, essuie tes doigts blancs. Un trait de craie sèche sur le ciment. Un trait de craie sèche sur le ciment, net.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le long du blanc, l'avion glisse jusqu'à la porte. Tu as tenu, j'ai tracé. Le pneu n'a plus mangé la piste. Tes mains ont laissé la piste. On rentre, essuie tes doigts blancs. Un trait de craie sèche sous les &lt;emphasis&gt;guidon&lt;/emphasis&gt;s. Un trait de craie sèche sur le ciment, net.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr"/>
@@ -13539,7 +13539,7 @@
 enfant-m|Le pneu n'a plus mangé la piste.
 papa|Tes mains ont laissé la piste.
 maman|On rentre, essuie tes doigts blancs.
-narrateur|Un trait de craie sèche sur le ciment.
+narrateur|Un trait de craie sèche sous les guidons.
 narrateur|Un trait de craie sèche sur le ciment, net.</t>
         </is>
       </c>
@@ -15803,17 +15803,17 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Un trait blanc cherche la porte. Près du battant, le vent pousse la poussière. Mila allonge le trait, trop tôt. J'ouvre grand, pour voir dehors ! Le trait s'envole en poussière, trop loin. Ma piste a volé ! Le blanc disparaît vers le seuil. Ici, le vent prend le trait. Il lui faut un air plus calme. Alors on fait comment ? Tu vois comment, avec lui ?</t>
+          <t>Un trait blanc cherche la porte. Près du battant, le vent pousse la poussière. Mila allonge le trait, trop tôt. J'ouvre grand, pour voir dehors ! Le trait s'envole en poussière, trop loin. Ma piste a volé ! Le blanc disparaît vers le seuil. Ici, le vent prend le trait. Sans le vent, le trait resterait. Alors on fait comment ? Tu vois comment, avec lui ?</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Un trait blanc cherche la porte. Près du battant, le &lt;emphasis level="moderate"&gt;vent&lt;/emphasis&gt; pousse la poussière. Mila allonge le trait, trop tôt. J'ouvre grand, pour voir dehors ! Le trait s'envole en poussière, trop loin. Ma piste a volé ! Le blanc disparaît vers le seuil. Ici, le vent prend le trait. Il lui faut un air plus calme. Alors on fait comment ? Tu vois comment, avec lui ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Un trait blanc cherche la porte. Près du battant, le &lt;emphasis level="moderate"&gt;vent&lt;/emphasis&gt; pousse la poussière. Mila allonge le trait, trop tôt. J'ouvre grand, pour voir dehors ! Le trait s'envole en poussière, trop loin. Ma piste a volé ! Le blanc disparaît vers le seuil. Ici, le vent prend le trait. Sans le vent, le trait resterait. Alors on fait comment ? Tu vois comment, avec lui ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Un trait blanc cherche la porte. Près du battant, le &lt;emphasis&gt;vent&lt;/emphasis&gt; pousse la poussière. Mila allonge le trait, trop tôt. J'ouvre grand, pour voir dehors ! Le trait s'envole en poussière, trop loin. Ma piste a volé ! Le blanc disparaît vers le seuil. Ici, le vent prend le trait. Il lui faut un air plus calme. Alors on fait comment ? Tu vois comment, avec lui ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Un trait blanc cherche la porte. Près du battant, le &lt;emphasis&gt;vent&lt;/emphasis&gt; pousse la poussière. Mila allonge le trait, trop tôt. J'ouvre grand, pour voir dehors ! Le trait s'envole en poussière, trop loin. Ma piste a volé ! Le blanc disparaît vers le seuil. Ici, le vent prend le trait. Sans le vent, le trait resterait. Alors on fait comment ? Tu vois comment, avec lui ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr"/>
@@ -15959,7 +15959,7 @@
 enfant-f|Ma piste a volé !
 narrateur|Le blanc disparaît vers le seuil.
 papa|Ici, le vent prend le trait.
-maman|Il lui faut un air plus calme.
+maman|Sans le vent, le trait resterait.
 enfant-f|Alors on fait comment ?
 papa|Tu vois comment, avec lui ?</t>
         </is>
@@ -17290,7 +17290,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17354,6 +17354,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>